<commit_message>
feat(similarity): Handle deltas in project date display
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_populate_similarities_body.xlsx
+++ b/tests/integration/test_data/test_populate_similarities_body.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58183B33-8A0A-4E46-81B6-F37B8B516C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF792DB8-575F-6849-954C-6063C98CC081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="34400" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -130,6 +130,15 @@
     <t>2024-10-24  22:07:37.0</t>
   </si>
   <si>
+    <t>Voici un autre corps qui va parler de Caisse d'allocation. Dans les nouveaux amendements on va changer un mot ou deux ou trois.</t>
+  </si>
+  <si>
+    <t>Voici un autre corps qui va parler de Caisse d'allocation. Dans les nouveaux amendements on va changer un mot ou deux ou plus mais ça matchera pas</t>
+  </si>
+  <si>
+    <t>La réponse est la suivante : foo2</t>
+  </si>
+  <si>
     <t>Réponse copiée de : PLFSS 2023
 Numéro d'amendement : 2
 Lecture : an 16
@@ -143,15 +152,6 @@
 Lecture : an 17
 Organe : Organe234
 Colonne similaire : Corps amdt</t>
-  </si>
-  <si>
-    <t>Voici un autre corps qui va parler de Caisse d'allocation. Dans les nouveaux amendements on va changer un mot ou deux ou trois.</t>
-  </si>
-  <si>
-    <t>Voici un autre corps qui va parler de Caisse d'allocation. Dans les nouveaux amendements on va changer un mot ou deux ou plus mais ça matchera pas</t>
-  </si>
-  <si>
-    <t>La réponse est la suivante : foo2</t>
   </si>
   <si>
     <t>Réponse copiée de : PLFSS 2023
@@ -180,21 +180,25 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -712,7 +716,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="19" t="s">
@@ -11732,7 +11736,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>26</v>
@@ -11776,13 +11780,13 @@
         <v>22</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>26</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>16</v>
@@ -11822,7 +11826,7 @@
         <v>26</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -11847,7 +11851,7 @@
         <v>18</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H5" s="6"/>
     </row>

</xml_diff>